<commit_message>
feat: update RSVP submission and wish handling
Add RSVP entry and public wishes, update submission logic in RsvpForm, and refine wish section event listeners to ensure real-time UI synchronization.
</commit_message>
<xml_diff>
--- a/public/wedding-rsvps.xlsx
+++ b/public/wedding-rsvps.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -469,9 +469,38 @@
         <v>Mubarak to the lovely couple!</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-09-26T16:10:35.710Z</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Dr. Salman Qureshi</v>
+      </c>
+      <c r="D3" t="str">
+        <v>+91 98765 43210</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Confirmed (Attending)</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="G3" t="str">
+        <v>nikah</v>
+      </c>
+      <c r="H3" t="str">
+        <v>None specified</v>
+      </c>
+      <c r="I3" t="str">
+        <v>May Allah bless this union with tranquility, eternal love, and prosperity. Congratulations to Basit &amp; Ambiya!</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -513,7 +542,7 @@
         <v>Total RSVP Responses</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -521,7 +550,7 @@
         <v>Confirmed Attending Responses</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -529,7 +558,7 @@
         <v>Total Guests (Heads)</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -537,7 +566,7 @@
         <v>Last Updated</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-09-25T19:04:05.327Z</v>
+        <v>2026-09-26T16:10:35.712Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(admin): implement RSVP and wish deletion
Add backend endpoint to remove RSVP/wish records and update the admin dashboard to allow direct management of guest wishes and RSVPs.
</commit_message>
<xml_diff>
--- a/public/wedding-rsvps.xlsx
+++ b/public/wedding-rsvps.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I2"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -469,38 +469,9 @@
         <v>Mubarak to the lovely couple!</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>2026-09-26T16:10:35.710Z</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Dr. Salman Qureshi</v>
-      </c>
-      <c r="D3" t="str">
-        <v>+91 98765 43210</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Confirmed (Attending)</v>
-      </c>
-      <c r="F3">
-        <v>2</v>
-      </c>
-      <c r="G3" t="str">
-        <v>nikah</v>
-      </c>
-      <c r="H3" t="str">
-        <v>None specified</v>
-      </c>
-      <c r="I3" t="str">
-        <v>May Allah bless this union with tranquility, eternal love, and prosperity. Congratulations to Basit &amp; Ambiya!</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -542,7 +513,7 @@
         <v>Total RSVP Responses</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -550,7 +521,7 @@
         <v>Confirmed Attending Responses</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -558,7 +529,7 @@
         <v>Total Guests (Heads)</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -566,7 +537,7 @@
         <v>Last Updated</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-09-26T16:10:35.712Z</v>
+        <v>2026-09-26T16:34:20.092Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>